<commit_message>
try to fix render prob
</commit_message>
<xml_diff>
--- a/data/Ingredient conflicts.xlsx
+++ b/data/Ingredient conflicts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yuyuanzhengjack/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9A9F002-7C47-4248-B081-346AC330E18E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01BC4413-A868-6940-8357-F9889044D63B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11540" yWindow="5440" windowWidth="28100" windowHeight="17360" xr2:uid="{44635FB0-5F1C-2C45-A6EE-0BBCDCFC00D0}"/>
   </bookViews>
@@ -104,94 +104,97 @@
     <t>Retinoids </t>
   </si>
   <si>
+    <t>Low-pH Niacinamide </t>
+  </si>
+  <si>
+    <t>Physical Exfoliants</t>
+  </si>
+  <si>
+    <t>Chemical Exfoliants</t>
+  </si>
+  <si>
+    <t>Copper Peptides</t>
+  </si>
+  <si>
+    <t>Photosensitizing Acids</t>
+  </si>
+  <si>
+    <t>High-concentration Alkalis</t>
+  </si>
+  <si>
+    <t>Peptides</t>
+  </si>
+  <si>
+    <t>SLES/SLS Harsh Surfactants</t>
+  </si>
+  <si>
+    <t>High-concentration Benzoyl Peroxide</t>
+  </si>
+  <si>
+    <t>High-concentration Salicylic Acid</t>
+  </si>
+  <si>
+    <t>Incompatible Vitamin E Formulations</t>
+  </si>
+  <si>
+    <t>Fragrance-rich Essential Oils</t>
+  </si>
+  <si>
+    <t>High-content Alcohol</t>
+  </si>
+  <si>
+    <t>High-molecular-weight Hyaluronic Acid </t>
+  </si>
+  <si>
+    <t>Silicone-heavy Occlusives</t>
+  </si>
+  <si>
+    <t>UV Filter Sunscreens</t>
+  </si>
+  <si>
+    <t>Unstable Antioxidants</t>
+  </si>
+  <si>
+    <t>Formaldehyde-releasing Preservatives</t>
+  </si>
+  <si>
+    <t>Sulfites</t>
+  </si>
+  <si>
+    <t>alcohol</t>
+  </si>
+  <si>
+    <t>protein</t>
+  </si>
+  <si>
+    <t>nicotinamid</t>
+  </si>
+  <si>
+    <t>vitamin C</t>
+  </si>
+  <si>
+    <t>nicotinamide </t>
+  </si>
+  <si>
+    <t>salicylic acid</t>
+  </si>
+  <si>
+    <t>retinol</t>
+  </si>
+  <si>
+    <t>fruit acid</t>
+  </si>
+  <si>
     <t>Pure Vitamin C (Ascorbic Acid) </t>
-  </si>
-  <si>
-    <t>Low-pH Niacinamide </t>
-  </si>
-  <si>
-    <t>Physical Exfoliants</t>
-  </si>
-  <si>
-    <t>Chemical Exfoliants</t>
-  </si>
-  <si>
-    <t>Copper Peptides</t>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>citrus/Lavender Essential Oils</t>
-  </si>
-  <si>
-    <t>Photosensitizing Acids</t>
-  </si>
-  <si>
-    <t>High-concentration Acids (pH &lt; 3.5)</t>
-  </si>
-  <si>
-    <t>High-concentration Alkalis</t>
-  </si>
-  <si>
-    <t>Peptides</t>
-  </si>
-  <si>
-    <t>SLES/SLS Harsh Surfactants</t>
-  </si>
-  <si>
-    <t>High-concentration Benzoyl Peroxide</t>
-  </si>
-  <si>
-    <t>High-concentration Salicylic Acid</t>
-  </si>
-  <si>
-    <t>Incompatible Vitamin E Formulations</t>
-  </si>
-  <si>
-    <t>Fragrance-rich Essential Oils</t>
-  </si>
-  <si>
-    <t>High-content Alcohol</t>
-  </si>
-  <si>
-    <t>High-molecular-weight Hyaluronic Acid </t>
-  </si>
-  <si>
-    <t>Silicone-heavy Occlusives</t>
-  </si>
-  <si>
-    <t>UV Filter Sunscreens</t>
-  </si>
-  <si>
-    <t>Unstable Antioxidants</t>
-  </si>
-  <si>
-    <t>Formaldehyde-releasing Preservatives</t>
-  </si>
-  <si>
-    <t>Sulfites</t>
-  </si>
-  <si>
-    <t>alcohol</t>
-  </si>
-  <si>
-    <t>protein</t>
-  </si>
-  <si>
-    <t>nicotinamid</t>
-  </si>
-  <si>
-    <t>vitamin C</t>
-  </si>
-  <si>
-    <t>nicotinamide </t>
-  </si>
-  <si>
-    <t>salicylic acid</t>
-  </si>
-  <si>
-    <t>retinol</t>
-  </si>
-  <si>
-    <t>fruit acid</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>High-concentration Acids</t>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -807,10 +810,10 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -823,10 +826,10 @@
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -834,39 +837,39 @@
         <v>4</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="2" t="s">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="2" t="s">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -874,7 +877,7 @@
         <v>4</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -882,7 +885,7 @@
         <v>5</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -890,63 +893,63 @@
         <v>8</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="44" spans="1:2">

</xml_diff>